<commit_message>
Akquise-Liste Kleidung: 30 kleine deutsche Mode-Shops
Gleiches Format wie die Supplement-/Kosmetik-Liste: Kontaktdaten,
Quelle, Produkte, Spalten zum Aussortieren und Nachrichtenentwürfe.
Außerdem in beiden Listen die Produktsätze der Nachrichten
grammatikalisch vervollständigt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfN8B2GjhuL3FjP6D8iqdr
</commit_message>
<xml_diff>
--- a/akquise/shops-supplements-kosmetik.xlsx
+++ b/akquise/shops-supplements-kosmetik.xlsx
@@ -2507,7 +2507,7 @@
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Hallo liebes Team von a&amp;o FEEL THE LIFE GbR,
-ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – eure veganen Haarpflege- und Stylingprodukte – und dass ihr plastikfrei im Recyclingkarton verschickt.
+ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – eure veganen Haarpflege- und Stylingprodukte – und dass ihr plastikfrei im Recyclingkarton verschickt – das gefällt mir sehr.
 Wir übernehmen für kleine Shops das Lagern, Verpacken und Verschicken der Bestellungen. So habt ihr mehr Zeit für eure Haarpflege-Linie, und eure Kunden bekommen ihre Pakete trotzdem schnell und liebevoll verpackt.
 Hättet ihr Lust auf ein kurzes, unverbindliches Gespräch (10 Minuten reichen)?
 Viele Grüße
@@ -2631,7 +2631,7 @@
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Hallo liebes Team von Seifenmanufaktur Würfel,
-ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – eure Natur-Haar- und Körperseifen vom Fuß der Zugspitze, in Kleinserien und sogar individuell auf Wunsch.
+ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – eure Natur-Haar- und Körperseifen vom Fuß der Zugspitze, in Kleinserien und sogar individuell auf Wunsch – das gefällt mir sehr.
 Wir übernehmen für kleine Shops das Lagern, Verpacken und Verschicken der Bestellungen. So habt ihr mehr Zeit für das Seifenmachen, und eure Kunden bekommen ihre Pakete trotzdem schnell und liebevoll verpackt.
 Hättet ihr Lust auf ein kurzes, unverbindliches Gespräch (10 Minuten reichen)?
 Viele Grüße
@@ -2755,7 +2755,7 @@
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Hallo liebes Team von be green – be better,
-ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – euer nachhaltiges Naturkosmetik-Sortiment – und dass man bei euch in Langenfeld sogar abholen kann.
+ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – euer nachhaltiges Naturkosmetik-Sortiment – und dass man bei euch in Langenfeld sogar abholen kann – das gefällt mir sehr.
 Wir übernehmen für kleine Shops das Lagern, Verpacken und Verschicken der Bestellungen. So habt ihr mehr Zeit für euren Shop und eure Kunden, und eure Kunden bekommen ihre Pakete trotzdem schnell und liebevoll verpackt.
 Hättet ihr Lust auf ein kurzes, unverbindliches Gespräch (10 Minuten reichen)?
 Viele Grüße
@@ -2972,7 +2972,7 @@
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Hallo liebes Team von Naturherz,
-ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – euer Sortiment an bio-zertifizierten Nahrungsergänzungsmitteln und Naturkosmetik.
+ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – euer Sortiment an bio-zertifizierten Nahrungsergänzungsmitteln und Naturkosmetik – das gefällt mir sehr.
 Wir übernehmen für kleine Shops das Lagern, Verpacken und Verschicken der Bestellungen. So habt ihr mehr Zeit für Beratung und Sortiment, und eure Kunden bekommen ihre Pakete trotzdem schnell und liebevoll verpackt.
 Hättet ihr Lust auf ein kurzes, unverbindliches Gespräch (10 Minuten reichen)?
 Viele Grüße
@@ -3158,7 +3158,7 @@
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Hallo liebes Team von livQ AG,
-ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – eure Nahrungsergänzungsmittel, die ihr auch an Apotheken und Therapeuten liefert.
+ich bin [DEIN NAME] von Packmotin. Ich habe mir euren Shop angeschaut – eure Nahrungsergänzungsmittel, die ihr auch an Apotheken und Therapeuten liefert – das gefällt mir sehr.
 Wir übernehmen für kleine Shops das Lagern, Verpacken und Verschicken der Bestellungen. So habt ihr mehr Zeit für Fachhandel und Kunden, und eure Kunden bekommen ihre Pakete trotzdem schnell und liebevoll verpackt.
 Hättet ihr Lust auf ein kurzes, unverbindliches Gespräch (10 Minuten reichen)?
 Viele Grüße

</xml_diff>

<commit_message>
Akquise: Meina Naturkosmetik hat Interesse gemeldet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfN8B2GjhuL3FjP6D8iqdr
</commit_message>
<xml_diff>
--- a/akquise/shops-supplements-kosmetik.xlsx
+++ b/akquise/shops-supplements-kosmetik.xlsx
@@ -42,7 +42,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -88,6 +93,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1109,61 +1120,69 @@
       <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Meina Naturkosmetik GbR</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Kosmetik</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>10317 Berlin</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>https://meina-naturkosmetik.de</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>0163 9257939</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>office@meina-naturkosmetik.de</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>https://www.lifeverde.de/gruene-unternehmen/naturkosmetik/meina/kontakt</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>Zertifizierte Naturkosmetik</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>GbR, 1–10 Mitarbeiter</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Rückmeldung</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>28.10.2026: hat Interesse gemeldet – nächster Schritt: Gespräch vereinbaren</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">

</xml_diff>